<commit_message>
feat: pass referral facility to task content for diabetes and hypertension forms
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/ncd_diabetes_referral.xlsx
+++ b/config/demo/forms/app/ncd_diabetes_referral.xlsx
@@ -339,7 +339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -393,17 +393,17 @@
           <t>readonly</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>constraint</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>constraint_message</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>default</t>
         </is>
@@ -713,141 +713,121 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>inputs</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>t_referral_facility</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>referral</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Diabetes PHC Referral</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>inputs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>glucose_note</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>**Previous Rapid Glucose Reading:** ${t_rapid_glucose} mg/dL</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>facility_label</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>if(${t_referral_facility} = 'phc', 'Primary Health Center', if(${t_referral_facility} = 'chc', 'Community Health Center', if(${t_referral_facility} = 'dh', 'District Hospital', 'PHC')))</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>phc_visited</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Did the patient visit the PHC?</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Diabetes ${facility_label} Referral</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>willing_to_visit</t>
+          <t>glucose_note</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Is the patient willing to visit the PHC?</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>${phc_visited} = 'no'</t>
+          <t>**Previous Rapid Glucose Reading:** ${t_rapid_glucose} mg/dL</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>not_willing_note</t>
+          <t>phc_visited</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Patient is not willing to visit PHC.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'no'</t>
+          <t>Did the patient visit the ${facility_label}?</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>phc_visit_date</t>
+          <t>willing_to_visit</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>When will the patient visit the PHC?</t>
+          <t>Is the patient willing to visit the ${facility_label}?</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -857,56 +837,71 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'yes'</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>. &gt;= today()</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Please select today or a future date.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>today()</t>
+          <t>${phc_visited} = 'no'</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>t_phc_visited</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>${phc_visited}</t>
+          <t>not_willing_note</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Patient is not willing to visit ${facility_label}.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'no'</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>t_willing_to_visit</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>${willing_to_visit}</t>
+          <t>phc_visit_date</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>When will the patient visit the ${facility_label}?</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'yes'</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>. &gt;= today()</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Please select today or a future date.</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>today()</t>
         </is>
       </c>
     </row>
@@ -918,24 +913,29 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>t_phc_visit_date</t>
+          <t>t_phc_visited</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>${phc_visit_date}</t>
+          <t>${phc_visited}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>t_willing_to_visit</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>${willing_to_visit}</t>
         </is>
       </c>
     </row>
@@ -947,27 +947,56 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>form_submit_timestamp_iso</t>
+          <t>t_phc_visit_date</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+          <t>${phc_visit_date}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>form_submit_timestamp_iso</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>form_submit_timestamp_display</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>format-date-time(now(), '%e-%b-%Y %H:%M:%S')</t>
         </is>
@@ -986,7 +1015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -1037,6 +1066,57 @@
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ncd_referral_facility</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>phc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Primary Health Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ncd_referral_facility</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>chc</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Community Health Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ncd_referral_facility</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>dh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>District Hospital</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update NCD referral tasks to use explicit report IDs for improved resolution tracking and form linkage
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/ncd_diabetes_referral.xlsx
+++ b/config/demo/forms/app/ncd_diabetes_referral.xlsx
@@ -339,7 +339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="M1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -557,27 +557,27 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>user</t>
+    <row r="11" ht="15" customHeight="1" s="9">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>ncd_source_id</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>user</t>
         </is>
       </c>
     </row>
@@ -589,58 +589,43 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>name</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>phone</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>user</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>_id</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Patient's Name</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>select-contact type-patient</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
+          <t>contact</t>
         </is>
       </c>
     </row>
@@ -652,17 +637,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>patient_id</t>
+          <t>_id</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Medic ID</t>
+          <t>Patient's Name</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>select-contact type-patient</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
@@ -674,12 +664,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Patient Name</t>
+          <t>Medic ID</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -691,126 +681,126 @@
     <row r="19" ht="15" customHeight="1" s="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>string</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>hidden</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>t_rapid_glucose</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="1">
-      <c r="A21" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="1">
+      <c r="A22" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>t_referral_facility</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="1">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>inputs</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="1">
-      <c r="A23" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="1">
+      <c r="A24" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>facility_label</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>if(${t_referral_facility} = 'phc', 'Primary Health Center', if(${t_referral_facility} = 'chc', 'Community Health Center', if(${t_referral_facility} = 'dh', 'District Hospital', 'PHC')))</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>referral</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Diabetes ${facility_label} Referral</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>glucose_note</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>**Previous Rapid Glucose Reading:** ${t_rapid_glucose} mg/dL</t>
+          <t>Diabetes ${facility_label} Referral</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>phc_visited</t>
+          <t>glucose_note</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Did the patient visit the ${facility_label}?</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>**Previous Rapid Glucose Reading:** ${t_rapid_glucose} mg/dL</t>
         </is>
       </c>
     </row>
@@ -822,120 +812,125 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>willing_to_visit</t>
+          <t>phc_visited</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Is the patient willing to visit the ${facility_label}?</t>
+          <t>Did the patient visit the ${facility_label}?</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>yes</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>${phc_visited} = 'no'</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>not_willing_note</t>
+          <t>willing_to_visit</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Patient is not willing to visit ${facility_label}.</t>
+          <t>Is the patient willing to visit the ${facility_label}?</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'no'</t>
+          <t>${phc_visited} = 'no'</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>phc_visit_date</t>
+          <t>not_willing_note</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>When will the patient visit the ${facility_label}?</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Patient is not willing to visit ${facility_label}.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'yes'</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>. &gt;= today()</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>Please select today or a future date.</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>today()</t>
+          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'no'</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>phc_visit_date</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>When will the patient visit the ${facility_label}?</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>${phc_visited} = 'no' and ${willing_to_visit} = 'yes'</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>. &gt;= today()</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Please select today or a future date.</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>t_phc_visited</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>${phc_visited}</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>t_willing_to_visit</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>${willing_to_visit}</t>
         </is>
       </c>
     </row>
@@ -947,41 +942,41 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>t_phc_visit_date</t>
+          <t>t_willing_to_visit</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>${phc_visit_date}</t>
+          <t>${willing_to_visit}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>t_phc_visit_date</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>${phc_visit_date}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>form_submit_timestamp_iso</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+          <t>referral</t>
         </is>
       </c>
     </row>
@@ -993,10 +988,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>form_submit_timestamp_iso</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
           <t>form_submit_timestamp_display</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>format-date-time(now(), '%e-%b-%Y %H:%M:%S')</t>
         </is>

</xml_diff>